<commit_message>
Actualiza portafolio 2026-06-18 16:40 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="288">
   <si>
     <t xml:space="preserve"> 50001533 - GESVIAL</t>
   </si>
@@ -4516,7 +4516,7 @@
         <v>46184.68921728009</v>
       </c>
       <c r="D52" s="5">
-        <v>46184.689458333334</v>
+        <v>46191.68718039352</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>205</v>
@@ -4525,9 +4525,11 @@
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H52" s="6"/>
+        <v>197</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>198</v>
+      </c>
       <c r="I52" s="5">
         <v>46188</v>
       </c>
@@ -4567,7 +4569,7 @@
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46185.70285011574</v>
+        <v>46191.687177245374</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>207</v>
@@ -4576,9 +4578,11 @@
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H53" s="9"/>
+        <v>197</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>198</v>
+      </c>
       <c r="I53" s="8">
         <v>46188</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>46184.69000751157</v>
       </c>
       <c r="D54" s="5">
-        <v>46184.69000853009</v>
+        <v>46191.6871738426</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>209</v>
@@ -4629,9 +4633,11 @@
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H54" s="6"/>
+        <v>197</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>198</v>
+      </c>
       <c r="I54" s="5">
         <v>46188</v>
       </c>
@@ -4673,7 +4679,7 @@
         <v>46184.69031962963</v>
       </c>
       <c r="D55" s="8">
-        <v>46184.69032116898</v>
+        <v>46191.687168993056</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>211</v>
@@ -4682,9 +4688,11 @@
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H55" s="9"/>
+        <v>197</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>198</v>
+      </c>
       <c r="I55" s="8">
         <v>46188</v>
       </c>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-21 16:22 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -4261,9 +4261,11 @@
       <c r="B48" s="5">
         <v>46118.662263819446</v>
       </c>
-      <c r="C48" s="6"/>
+      <c r="C48" s="5">
+        <v>46194.056337268514</v>
+      </c>
       <c r="D48" s="5">
-        <v>46193.56241145833</v>
+        <v>46194.05633912037</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>189</v>
@@ -4721,9 +4723,11 @@
       <c r="B56" s="5">
         <v>46118.66228488426</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46194.05632121528</v>
+      </c>
       <c r="D56" s="5">
-        <v>46193.56235371528</v>
+        <v>46194.05632325231</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 21:56 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -251,9 +251,6 @@
     <t>Ingenieria Servicios:,Embalaje</t>
   </si>
   <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
     <t>1213955236952399</t>
   </si>
   <si>
@@ -429,6 +426,9 @@
   </si>
   <si>
     <t>Fabricación Alabe - OT4285,Generación OC Alabe - OT4285</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
   </si>
   <si>
     <t>1213973327836153</t>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46129.57130488426</v>
+        <v>46196.895724664355</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -2065,9 +2065,11 @@
       <c r="B12" s="5">
         <v>46118.66203578704</v>
       </c>
-      <c r="C12" s="6"/>
+      <c r="C12" s="5">
+        <v>46196.89571644676</v>
+      </c>
       <c r="D12" s="5">
-        <v>46195.52671909722</v>
+        <v>46196.89571872685</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -2112,18 +2114,18 @@
         <v>46191</v>
       </c>
       <c r="S12" s="6">
-        <v>0</v>
-      </c>
-      <c r="T12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="U12" s="11" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="U12" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B13" s="8">
         <v>46118.66186076389</v>
@@ -2135,7 +2137,7 @@
         <v>46193.561794629626</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2159,7 +2161,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2172,7 +2174,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46118.66204173611</v>
@@ -2184,7 +2186,7 @@
         <v>46191.77226219907</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2205,19 +2207,19 @@
         <v>26</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="5">
         <v>46107</v>
@@ -2237,7 +2239,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B15" s="8">
         <v>46118.66204752315</v>
@@ -2249,7 +2251,7 @@
         <v>46191.77226225694</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2270,19 +2272,19 @@
         <v>26</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="8">
         <v>46114</v>
@@ -2302,7 +2304,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46118.66205295139</v>
@@ -2314,7 +2316,7 @@
         <v>46191.7722621412</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2335,19 +2337,19 @@
         <v>26</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q16" s="5">
         <v>46114</v>
@@ -2367,7 +2369,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" s="8">
         <v>46118.6618661574</v>
@@ -2379,7 +2381,7 @@
         <v>46184.72974401621</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>25</v>
@@ -2403,7 +2405,7 @@
         <v>26</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>26</v>
@@ -2416,7 +2418,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="5">
         <v>46118.66206653936</v>
@@ -2428,7 +2430,7 @@
         <v>46129.56236072916</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
@@ -2449,19 +2451,19 @@
         <v>26</v>
       </c>
       <c r="L18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="O18" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="Q18" s="5">
         <v>46118</v>
@@ -2481,7 +2483,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="8">
         <v>46118.66207174768</v>
@@ -2493,7 +2495,7 @@
         <v>46129.56236737268</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
@@ -2514,19 +2516,19 @@
         <v>26</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="8">
         <v>46111</v>
@@ -2546,7 +2548,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20" s="5">
         <v>46118.66207709491</v>
@@ -2558,7 +2560,7 @@
         <v>46129.57135429398</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2579,19 +2581,19 @@
         <v>26</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>51</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q20" s="5">
         <v>46112</v>
@@ -2611,7 +2613,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21" s="8">
         <v>46118.66208231481</v>
@@ -2623,16 +2625,16 @@
         <v>46183.880102916664</v>
       </c>
       <c r="E21" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>92</v>
-      </c>
       <c r="H21" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I21" s="8">
         <v>46115</v>
@@ -2650,13 +2652,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q21" s="8">
         <v>46118</v>
@@ -2671,12 +2673,12 @@
         <v>55</v>
       </c>
       <c r="U21" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B22" s="5">
         <v>46118.662087523146</v>
@@ -2688,16 +2690,16 @@
         <v>46183.888251435186</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="I22" s="5">
         <v>46150</v>
@@ -2715,13 +2717,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O22" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="P22" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="P22" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="Q22" s="5">
         <v>46153</v>
@@ -2736,12 +2738,12 @@
         <v>32</v>
       </c>
       <c r="U22" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B23" s="8">
         <v>46118.66187195602</v>
@@ -2753,7 +2755,7 @@
         <v>46184.686248067126</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>25</v>
@@ -2777,7 +2779,7 @@
         <v>26</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P23" s="9" t="s">
         <v>26</v>
@@ -2790,7 +2792,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="5">
         <v>46118.662093692124</v>
@@ -2802,16 +2804,16 @@
         <v>46182.676449293984</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G24" s="6" t="s">
+      <c r="H24" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I24" s="5">
         <v>46119</v>
@@ -2829,13 +2831,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="5">
         <v>46232</v>
@@ -2850,7 +2852,7 @@
         <v>32</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -2873,10 +2875,10 @@
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I25" s="8">
         <v>46119</v>
@@ -2894,10 +2896,10 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>111</v>
@@ -2928,10 +2930,10 @@
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I26" s="5">
         <v>46121</v>
@@ -2949,7 +2951,7 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>110</v>
@@ -2983,10 +2985,10 @@
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I27" s="8">
         <v>46111</v>
@@ -3004,13 +3006,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O27" s="9" t="s">
         <v>117</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q27" s="8">
         <v>46188</v>
@@ -3025,7 +3027,7 @@
         <v>32</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3048,10 +3050,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I28" s="5">
         <v>46111</v>
@@ -3072,7 +3074,7 @@
         <v>116</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>120</v>
@@ -3086,7 +3088,7 @@
         <v>32</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3109,10 +3111,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I29" s="8">
         <v>46120</v>
@@ -3147,7 +3149,7 @@
         <v>32</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3170,10 +3172,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I30" s="5">
         <v>46119</v>
@@ -3191,13 +3193,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>126</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q30" s="5">
         <v>46167</v>
@@ -3212,7 +3214,7 @@
         <v>32</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3235,10 +3237,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I31" s="8">
         <v>46119</v>
@@ -3259,7 +3261,7 @@
         <v>125</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P31" s="9" t="s">
         <v>129</v>
@@ -3273,7 +3275,7 @@
         <v>32</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3296,10 +3298,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I32" s="5">
         <v>46121</v>
@@ -3334,7 +3336,7 @@
         <v>32</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3357,10 +3359,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I33" s="8">
         <v>46112</v>
@@ -3378,13 +3380,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O33" s="9" t="s">
         <v>135</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q33" s="8">
         <v>46254</v>
@@ -3399,7 +3401,7 @@
         <v>32</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3422,10 +3424,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I34" s="5">
         <v>46112</v>
@@ -3446,7 +3448,7 @@
         <v>134</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P34" s="6" t="s">
         <v>138</v>
@@ -3460,7 +3462,7 @@
         <v>32</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3483,10 +3485,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="I35" s="8">
         <v>46133</v>
@@ -3521,7 +3523,7 @@
         <v>32</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -3544,10 +3546,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="I36" s="5">
         <v>46133</v>
@@ -3582,7 +3584,7 @@
         <v>32</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -3626,13 +3628,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O37" s="9" t="s">
         <v>131</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q37" s="8">
         <v>46170</v>
@@ -3647,7 +3649,7 @@
         <v>32</v>
       </c>
       <c r="U37" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -3694,7 +3696,7 @@
         <v>146</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>151</v>
@@ -3708,7 +3710,7 @@
         <v>32</v>
       </c>
       <c r="U38" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -3769,7 +3771,7 @@
         <v>32</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -3863,7 +3865,7 @@
         <v>155</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P41" s="9" t="s">
         <v>161</v>
@@ -3963,7 +3965,7 @@
         <v>46134.80040836806</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
@@ -4072,7 +4074,7 @@
         <v>32</v>
       </c>
       <c r="U44" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -4186,7 +4188,7 @@
         <v>32</v>
       </c>
       <c r="U46" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -4251,7 +4253,7 @@
         <v>32</v>
       </c>
       <c r="U47" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -4365,7 +4367,7 @@
         <v>32</v>
       </c>
       <c r="U49" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -4430,7 +4432,7 @@
         <v>32</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4715,7 +4717,7 @@
         <v>32</v>
       </c>
       <c r="U55" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4829,7 +4831,7 @@
         <v>32</v>
       </c>
       <c r="U57" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -4894,7 +4896,7 @@
         <v>32</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -4959,7 +4961,7 @@
         <v>32</v>
       </c>
       <c r="U59" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5024,7 +5026,7 @@
         <v>32</v>
       </c>
       <c r="U60" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5096,10 +5098,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I62" s="5">
         <v>46210</v>
@@ -5138,7 +5140,7 @@
         <v>32</v>
       </c>
       <c r="U62" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5161,10 +5163,10 @@
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I63" s="8">
         <v>46259</v>
@@ -5203,7 +5205,7 @@
         <v>32</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5226,10 +5228,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I64" s="5">
         <v>46261</v>
@@ -5268,7 +5270,7 @@
         <v>32</v>
       </c>
       <c r="U64" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5291,10 +5293,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I65" s="8">
         <v>46265</v>
@@ -5333,7 +5335,7 @@
         <v>32</v>
       </c>
       <c r="U65" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5356,10 +5358,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="5">
@@ -5396,7 +5398,7 @@
         <v>32</v>
       </c>
       <c r="U66" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5417,10 +5419,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I67" s="8">
         <v>46269</v>
@@ -5459,7 +5461,7 @@
         <v>32</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5567,7 +5569,7 @@
         <v>32</v>
       </c>
       <c r="U69" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5579,7 +5581,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46196.57543765046</v>
+        <v>46196.89572584491</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>255</v>
@@ -5588,10 +5590,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5628,7 +5630,7 @@
         <v>32</v>
       </c>
       <c r="U70" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5689,7 +5691,7 @@
         <v>32</v>
       </c>
       <c r="U71" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5750,7 +5752,7 @@
         <v>32</v>
       </c>
       <c r="U72" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5860,7 +5862,7 @@
         <v>32</v>
       </c>
       <c r="U74" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5923,7 +5925,7 @@
         <v>32</v>
       </c>
       <c r="U75" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6033,7 +6035,7 @@
         <v>32</v>
       </c>
       <c r="U77" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6096,7 +6098,7 @@
         <v>32</v>
       </c>
       <c r="U78" s="11" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 19:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -5477,7 +5477,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46196.92306695602</v>
+        <v>46203.815654895836</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>247</v>
@@ -5522,9 +5522,11 @@
       <c r="B69" s="8">
         <v>46118.662431770834</v>
       </c>
-      <c r="C69" s="9"/>
+      <c r="C69" s="8">
+        <v>46203.81564377315</v>
+      </c>
       <c r="D69" s="8">
-        <v>46203.57157956019</v>
+        <v>46203.8156465625</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>250</v>
@@ -5585,7 +5587,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46196.89572584491</v>
+        <v>46203.81565671296</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>255</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-01 15:51 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -1953,9 +1953,11 @@
       <c r="B10" s="5">
         <v>46118.66185618055</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46204.65215401621</v>
+      </c>
       <c r="D10" s="5">
-        <v>46196.895724664355</v>
+        <v>46204.65215631944</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>48</v>
@@ -3781,9 +3783,11 @@
       <c r="B40" s="5">
         <v>46118.662220972226</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46204.65218209491</v>
+      </c>
       <c r="D40" s="5">
-        <v>46198.56946403935</v>
+        <v>46204.652183645834</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>155</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-05 01:25 Chile
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -2624,7 +2624,7 @@
         <v>46183.88010105324</v>
       </c>
       <c r="D21" s="8">
-        <v>46183.880102916664</v>
+        <v>46208.21006932871</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>90</v>
@@ -2669,7 +2669,7 @@
         <v>46115</v>
       </c>
       <c r="S21" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" s="11" t="s">
         <v>55</v>
@@ -2689,7 +2689,7 @@
         <v>46183.888051863425</v>
       </c>
       <c r="D22" s="5">
-        <v>46183.888251435186</v>
+        <v>46208.21011525463</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>95</v>
@@ -2734,7 +2734,7 @@
         <v>46150</v>
       </c>
       <c r="S22" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T22" s="10" t="s">
         <v>32</v>
@@ -2803,7 +2803,7 @@
         <v>46182.67644689815</v>
       </c>
       <c r="D24" s="5">
-        <v>46182.676449293984</v>
+        <v>46208.21003241898</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>104</v>
@@ -2848,7 +2848,7 @@
         <v>46119</v>
       </c>
       <c r="S24" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" s="10" t="s">
         <v>32</v>
@@ -2868,7 +2868,7 @@
         <v>46174.62568537037</v>
       </c>
       <c r="D25" s="8">
-        <v>46174.62568689814</v>
+        <v>46208.21094784723</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>110</v>
@@ -2908,7 +2908,9 @@
       </c>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
+      <c r="S25" s="9">
+        <v>1</v>
+      </c>
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
     </row>
@@ -2923,7 +2925,7 @@
         <v>46182.64328993055</v>
       </c>
       <c r="D26" s="5">
-        <v>46182.64329142361</v>
+        <v>46208.21109037037</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>113</v>
@@ -2963,7 +2965,9 @@
       </c>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="S26" s="6">
+        <v>1</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
     </row>
@@ -2978,7 +2982,7 @@
         <v>46182.641066956014</v>
       </c>
       <c r="D27" s="8">
-        <v>46182.64106920139</v>
+        <v>46208.209962824076</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>116</v>
@@ -3023,7 +3027,7 @@
         <v>46111</v>
       </c>
       <c r="S27" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T27" s="10" t="s">
         <v>32</v>
@@ -3043,7 +3047,7 @@
         <v>46174.626521666665</v>
       </c>
       <c r="D28" s="5">
-        <v>46174.62652314815</v>
+        <v>46208.21118949074</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>119</v>
@@ -3084,7 +3088,7 @@
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" s="10" t="s">
         <v>32</v>
@@ -3104,7 +3108,7 @@
         <v>46174.626630416664</v>
       </c>
       <c r="D29" s="8">
-        <v>46174.62663186343</v>
+        <v>46208.21130763889</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>122</v>
@@ -3145,7 +3149,7 @@
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
       <c r="S29" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T29" s="10" t="s">
         <v>32</v>
@@ -3165,7 +3169,7 @@
         <v>46184.68608144676</v>
       </c>
       <c r="D30" s="5">
-        <v>46184.68608324074</v>
+        <v>46208.20888993055</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>125</v>
@@ -3210,7 +3214,7 @@
         <v>46119</v>
       </c>
       <c r="S30" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T30" s="10" t="s">
         <v>32</v>
@@ -3230,7 +3234,7 @@
         <v>46184.68571903935</v>
       </c>
       <c r="D31" s="8">
-        <v>46184.68572081019</v>
+        <v>46208.211394502316</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>128</v>
@@ -3271,7 +3275,7 @@
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
       <c r="S31" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T31" s="10" t="s">
         <v>32</v>
@@ -3291,7 +3295,7 @@
         <v>46184.68578890046</v>
       </c>
       <c r="D32" s="5">
-        <v>46184.68579053241</v>
+        <v>46208.21147013889</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>131</v>
@@ -3332,7 +3336,7 @@
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T32" s="10" t="s">
         <v>32</v>
@@ -3417,7 +3421,7 @@
         <v>46134.79115269676</v>
       </c>
       <c r="D34" s="5">
-        <v>46169.823994363425</v>
+        <v>46208.211555636575</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>137</v>
@@ -3458,7 +3462,7 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T34" s="10" t="s">
         <v>32</v>
@@ -3478,7 +3482,7 @@
         <v>46155.90268767361</v>
       </c>
       <c r="D35" s="8">
-        <v>46169.82401586806</v>
+        <v>46208.21164188658</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>140</v>
@@ -3519,7 +3523,7 @@
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
       <c r="S35" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" s="10" t="s">
         <v>32</v>
@@ -3539,7 +3543,7 @@
         <v>46134.79119539352</v>
       </c>
       <c r="D36" s="5">
-        <v>46169.824036157406</v>
+        <v>46208.211714791665</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>143</v>
@@ -3580,7 +3584,7 @@
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" s="10" t="s">
         <v>32</v>
@@ -3600,7 +3604,7 @@
         <v>46184.686103796295</v>
       </c>
       <c r="D37" s="8">
-        <v>46184.68610523148</v>
+        <v>46208.208834942125</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>146</v>
@@ -3645,7 +3649,7 @@
         <v>46154</v>
       </c>
       <c r="S37" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T37" s="10" t="s">
         <v>32</v>
@@ -3665,7 +3669,7 @@
         <v>46184.53094861111</v>
       </c>
       <c r="D38" s="5">
-        <v>46184.53095076389</v>
+        <v>46208.21179649305</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>150</v>
@@ -3706,7 +3710,7 @@
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
       <c r="S38" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T38" s="10" t="s">
         <v>32</v>
@@ -3726,7 +3730,7 @@
         <v>46184.53162540509</v>
       </c>
       <c r="D39" s="8">
-        <v>46184.531626724536</v>
+        <v>46208.211892453706</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>151</v>
@@ -3767,7 +3771,7 @@
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
       <c r="S39" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T39" s="10" t="s">
         <v>32</v>
@@ -4029,7 +4033,7 @@
         <v>46198.5694571412</v>
       </c>
       <c r="D44" s="5">
-        <v>46198.56945943287</v>
+        <v>46208.20879145833</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>171</v>
@@ -4074,7 +4078,7 @@
         <v>46268</v>
       </c>
       <c r="S44" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T44" s="10" t="s">
         <v>32</v>
@@ -4143,7 +4147,7 @@
         <v>46184.68670658565</v>
       </c>
       <c r="D46" s="5">
-        <v>46184.686925347225</v>
+        <v>46208.20988328704</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>153</v>
@@ -4188,7 +4192,7 @@
         <v>46171</v>
       </c>
       <c r="S46" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T46" s="10" t="s">
         <v>32</v>
@@ -4208,7 +4212,7 @@
         <v>46184.6869659838</v>
       </c>
       <c r="D47" s="8">
-        <v>46184.68714663194</v>
+        <v>46208.20991337963</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>184</v>
@@ -4253,7 +4257,7 @@
         <v>46175</v>
       </c>
       <c r="S47" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T47" s="10" t="s">
         <v>32</v>
@@ -4322,7 +4326,7 @@
         <v>46184.687951203705</v>
       </c>
       <c r="D49" s="8">
-        <v>46184.687952719905</v>
+        <v>46208.210227986114</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>192</v>
@@ -4367,7 +4371,7 @@
         <v>46177</v>
       </c>
       <c r="S49" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T49" s="10" t="s">
         <v>32</v>
@@ -4387,7 +4391,7 @@
         <v>46193.56191304398</v>
       </c>
       <c r="D50" s="5">
-        <v>46193.561914942125</v>
+        <v>46208.210261203705</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>197</v>
@@ -4432,7 +4436,7 @@
         <v>46188</v>
       </c>
       <c r="S50" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T50" s="10" t="s">
         <v>32</v>
@@ -4672,7 +4676,7 @@
         <v>46193.56240042824</v>
       </c>
       <c r="D55" s="8">
-        <v>46193.562405625</v>
+        <v>46208.21032709491</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>209</v>
@@ -4717,7 +4721,7 @@
         <v>46206</v>
       </c>
       <c r="S55" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T55" s="10" t="s">
         <v>32</v>
@@ -4786,7 +4790,7 @@
         <v>46193.562345370374</v>
       </c>
       <c r="D57" s="8">
-        <v>46193.56234733797</v>
+        <v>46208.21036678241</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>215</v>
@@ -4831,7 +4835,7 @@
         <v>46168</v>
       </c>
       <c r="S57" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T57" s="10" t="s">
         <v>32</v>
@@ -4851,7 +4855,7 @@
         <v>46193.56197458333</v>
       </c>
       <c r="D58" s="5">
-        <v>46193.56197650463</v>
+        <v>46208.210472280094</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>58</v>
@@ -4896,7 +4900,7 @@
         <v>46189</v>
       </c>
       <c r="S58" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T58" s="10" t="s">
         <v>32</v>
@@ -4916,7 +4920,7 @@
         <v>46193.561984872686</v>
       </c>
       <c r="D59" s="8">
-        <v>46193.561986678236</v>
+        <v>46208.21047276621</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>220</v>
@@ -4961,7 +4965,7 @@
         <v>46233</v>
       </c>
       <c r="S59" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59" s="10" t="s">
         <v>32</v>
@@ -4981,7 +4985,7 @@
         <v>46193.56199724537</v>
       </c>
       <c r="D60" s="5">
-        <v>46193.56199886574</v>
+        <v>46208.210473217594</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>223</v>
@@ -5026,7 +5030,7 @@
         <v>46255</v>
       </c>
       <c r="S60" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T60" s="10" t="s">
         <v>32</v>
@@ -5095,7 +5099,7 @@
         <v>46193.61261344908</v>
       </c>
       <c r="D62" s="5">
-        <v>46196.921998854166</v>
+        <v>46208.21062993056</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>229</v>
@@ -5140,7 +5144,7 @@
         <v>46210</v>
       </c>
       <c r="S62" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T62" s="10" t="s">
         <v>32</v>
@@ -5160,7 +5164,7 @@
         <v>46193.6126587037</v>
       </c>
       <c r="D63" s="8">
-        <v>46193.61266056713</v>
+        <v>46208.21062945602</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>224</v>
@@ -5205,7 +5209,7 @@
         <v>46259</v>
       </c>
       <c r="S63" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T63" s="10" t="s">
         <v>32</v>
@@ -5225,7 +5229,7 @@
         <v>46193.61267944444</v>
       </c>
       <c r="D64" s="5">
-        <v>46193.61268100694</v>
+        <v>46208.21063037037</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>235</v>
@@ -5270,7 +5274,7 @@
         <v>46261</v>
       </c>
       <c r="S64" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T64" s="10" t="s">
         <v>32</v>
@@ -5290,7 +5294,7 @@
         <v>46193.61273716435</v>
       </c>
       <c r="D65" s="8">
-        <v>46193.61273954861</v>
+        <v>46208.21062888889</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>238</v>
@@ -5335,7 +5339,7 @@
         <v>46265</v>
       </c>
       <c r="S65" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T65" s="10" t="s">
         <v>32</v>
@@ -5355,7 +5359,7 @@
         <v>46193.765511875</v>
       </c>
       <c r="D66" s="5">
-        <v>46193.765518935186</v>
+        <v>46208.21062840278</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>174</v>
@@ -5398,7 +5402,7 @@
         <v>46267</v>
       </c>
       <c r="S66" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T66" s="10" t="s">
         <v>32</v>
@@ -5418,7 +5422,7 @@
         <v>46196.92346424768</v>
       </c>
       <c r="D67" s="8">
-        <v>46198.56946547454</v>
+        <v>46208.21062791666</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>244</v>
@@ -5463,7 +5467,7 @@
         <v>46269</v>
       </c>
       <c r="S67" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67" s="10" t="s">
         <v>32</v>
@@ -5530,7 +5534,7 @@
         <v>46203.81564377315</v>
       </c>
       <c r="D69" s="8">
-        <v>46204.900270983795</v>
+        <v>46208.21071721065</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>250</v>
@@ -5573,7 +5577,7 @@
         <v>46272</v>
       </c>
       <c r="S69" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T69" s="10" t="s">
         <v>32</v>
@@ -5593,7 +5597,7 @@
         <v>46204.89777927083</v>
       </c>
       <c r="D70" s="5">
-        <v>46204.90025034722</v>
+        <v>46208.210717662034</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>255</v>
@@ -5636,7 +5640,7 @@
         <v>46273</v>
       </c>
       <c r="S70" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T70" s="10" t="s">
         <v>32</v>
@@ -5656,7 +5660,7 @@
         <v>46196.9230577662</v>
       </c>
       <c r="D71" s="8">
-        <v>46204.900126967594</v>
+        <v>46208.210718125</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>259</v>
@@ -5699,7 +5703,7 @@
         <v>46274</v>
       </c>
       <c r="S71" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T71" s="10" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 17:37 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46209.53540731482</v>
+        <v>46209.72177900463</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>264</v>
@@ -5769,8 +5769,8 @@
       <c r="T72" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U72" s="11" t="s">
-        <v>108</v>
+      <c r="U72" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-17 13:45 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -4961,7 +4961,7 @@
         <v>46193.56199724537</v>
       </c>
       <c r="D60" s="5">
-        <v>46208.210473217594</v>
+        <v>46251.18919104167</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>223</v>
@@ -5008,8 +5008,8 @@
       <c r="S60" s="6">
         <v>1</v>
       </c>
-      <c r="T60" s="10" t="s">
-        <v>32</v>
+      <c r="T60" s="12" t="s">
+        <v>135</v>
       </c>
       <c r="U60" s="11" t="s">
         <v>107</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-25 13:53 UTC
</commit_message>
<xml_diff>
--- a/data/50001533 - GESVIAL.xlsx
+++ b/data/50001533 - GESVIAL.xlsx
@@ -776,34 +776,34 @@
     <t>Montaje motor</t>
   </si>
   <si>
+    <t>1213964538772999</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,RE-PINTADO,Montaje motor,Montaje Alabe,Montaje Rodete,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213955269755930</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>Montaje:,Montaje Alabe,Montaje Rodete,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213955269755950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revestimiento,Recepcion motor,Check planos </t>
+  </si>
+  <si>
+    <t>Montaje:,Pruebas FAT</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213964538772999</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,RE-PINTADO,Montaje motor,Montaje Alabe,Montaje Rodete,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213955269755930</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>Montaje:,Montaje Alabe,Montaje Rodete,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213955269755950</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revestimiento,Recepcion motor,Check planos </t>
-  </si>
-  <si>
-    <t>Montaje:,Pruebas FAT</t>
   </si>
   <si>
     <t>1213963540685278</t>
@@ -4961,7 +4961,7 @@
         <v>46193.56199724537</v>
       </c>
       <c r="D60" s="5">
-        <v>46251.18919104167</v>
+        <v>46259.20590515046</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>222</v>
@@ -5008,8 +5008,8 @@
       <c r="S60" s="6">
         <v>1</v>
       </c>
-      <c r="T60" s="12" t="s">
-        <v>224</v>
+      <c r="T60" s="11" t="s">
+        <v>55</v>
       </c>
       <c r="U60" s="11" t="s">
         <v>107</v>
@@ -5017,7 +5017,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B61" s="8">
         <v>46118.66236295139</v>
@@ -5029,7 +5029,7 @@
         <v>46204.900153703704</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>25</v>
@@ -5053,7 +5053,7 @@
         <v>26</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>26</v>
@@ -5066,7 +5066,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B62" s="5">
         <v>46118.66236873843</v>
@@ -5078,7 +5078,7 @@
         <v>46228.2021169213</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
@@ -5105,13 +5105,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>208</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Q62" s="5">
         <v>46227</v>
@@ -5131,7 +5131,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B63" s="8">
         <v>46118.662376064814</v>
@@ -5170,13 +5170,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O63" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="P63" s="9" t="s">
         <v>232</v>
-      </c>
-      <c r="P63" s="9" t="s">
-        <v>233</v>
       </c>
       <c r="Q63" s="8">
         <v>46260</v>
@@ -5188,7 +5188,7 @@
         <v>1</v>
       </c>
       <c r="T63" s="12" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="U63" s="11" t="s">
         <v>107</v>
@@ -5235,13 +5235,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>236</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q64" s="5">
         <v>46262</v>
@@ -5253,7 +5253,7 @@
         <v>1</v>
       </c>
       <c r="T64" s="12" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="U64" s="11" t="s">
         <v>107</v>
@@ -5270,7 +5270,7 @@
         <v>46193.61273716435</v>
       </c>
       <c r="D65" s="8">
-        <v>46223.807257754626</v>
+        <v>46259.1828917824</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>238</v>
@@ -5300,13 +5300,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O65" s="9" t="s">
         <v>239</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Q65" s="8">
         <v>46266</v>
@@ -5317,8 +5317,8 @@
       <c r="S65" s="9">
         <v>1</v>
       </c>
-      <c r="T65" s="10" t="s">
-        <v>32</v>
+      <c r="T65" s="12" t="s">
+        <v>233</v>
       </c>
       <c r="U65" s="11" t="s">
         <v>107</v>
@@ -5363,7 +5363,7 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>241</v>
@@ -5428,7 +5428,7 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O67" s="9" t="s">
         <v>170</v>

</xml_diff>